<commit_message>
Actualització PowerPoint i Burn-down
</commit_message>
<xml_diff>
--- a/documents/Sprint3/Burndownchart3.xlsx
+++ b/documents/Sprint3/Burndownchart3.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marcs\Downloads\ES\PRACTIQUES\ES23UAB431-02\documents\Sprint3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20A66209-D60C-4C1E-848C-94A5B4365297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64B8A5CD-30D1-4A62-B283-09E130A5E0B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="17472" windowHeight="10992" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20520" yWindow="-5505" windowWidth="20640" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BLANK - Simple Burndown Chart" sheetId="1" r:id="rId1"/>
@@ -58,9 +58,6 @@
     <t>PROJECT ID</t>
   </si>
   <si>
-    <t>Sprint 1</t>
-  </si>
-  <si>
     <t>Alejandro Ibarra Amaro</t>
   </si>
   <si>
@@ -87,6 +84,9 @@
   </si>
   <si>
     <t>BURNDOWN</t>
+  </si>
+  <si>
+    <t>Sprint 3</t>
   </si>
 </sst>
 </file>
@@ -136,10 +136,10 @@
       <name val="Century Gothic"/>
     </font>
     <font>
-      <u/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="10">
@@ -660,37 +660,37 @@
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>58</c:v>
+                  <c:v>57</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>53</c:v>
+                  <c:v>52</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>45</c:v>
+                  <c:v>43</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>37</c:v>
+                  <c:v>34</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>30</c:v>
+                  <c:v>26</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>25</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>16</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>12</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>0</c:v>
@@ -784,37 +784,37 @@
                   <c:v>60</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>60</c:v>
+                  <c:v>51</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>60</c:v>
+                  <c:v>41</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>60</c:v>
+                  <c:v>33</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>60</c:v>
+                  <c:v>19</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>60</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>60</c:v>
+                  <c:v>11</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>60</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>60</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>60</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>60</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>60</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1312,23 +1312,23 @@
     <row r="3" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A3" s="4"/>
       <c r="B3" s="28" t="s">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="C3" s="29"/>
       <c r="D3" s="29"/>
       <c r="E3" s="29"/>
       <c r="F3" s="30"/>
       <c r="G3" s="8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H3" s="9">
         <v>46090</v>
       </c>
       <c r="I3" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="J3" s="11" t="s">
         <v>8</v>
-      </c>
-      <c r="J3" s="11" t="s">
-        <v>9</v>
       </c>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
@@ -1378,22 +1378,22 @@
     <row r="5" spans="1:26" ht="69.75" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A5" s="3"/>
       <c r="B5" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="D5" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="13" t="s">
+      <c r="E5" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="F5" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="G5" s="16" t="s">
         <v>14</v>
-      </c>
-      <c r="G5" s="16" t="s">
-        <v>15</v>
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
@@ -1459,14 +1459,14 @@
         <v>1</v>
       </c>
       <c r="C7" s="18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7" s="19">
         <v>0</v>
       </c>
       <c r="E7" s="22">
         <f t="shared" ref="E7:F7" si="0">E6-C7</f>
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F7" s="23">
         <f t="shared" si="0"/>
@@ -1502,15 +1502,15 @@
         <v>5</v>
       </c>
       <c r="D8" s="19">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E8" s="22">
         <f t="shared" ref="E8:F8" si="1">E7-C8</f>
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F8" s="23">
         <f t="shared" si="1"/>
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
@@ -1539,18 +1539,18 @@
         <v>3</v>
       </c>
       <c r="C9" s="18">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D9" s="19">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E9" s="22">
         <f t="shared" ref="E9:F9" si="2">E8-C9</f>
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F9" s="23">
         <f t="shared" si="2"/>
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
@@ -1579,18 +1579,18 @@
         <v>4</v>
       </c>
       <c r="C10" s="18">
+        <v>9</v>
+      </c>
+      <c r="D10" s="19">
         <v>8</v>
-      </c>
-      <c r="D10" s="19">
-        <v>0</v>
       </c>
       <c r="E10" s="22">
         <f t="shared" ref="E10:F10" si="3">E9-C10</f>
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F10" s="23">
         <f t="shared" si="3"/>
-        <v>60</v>
+        <v>33</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
@@ -1619,18 +1619,18 @@
         <v>5</v>
       </c>
       <c r="C11" s="18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D11" s="19">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="E11" s="22">
         <f t="shared" ref="E11:F11" si="4">E10-C11</f>
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F11" s="23">
         <f t="shared" si="4"/>
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
@@ -1662,15 +1662,15 @@
         <v>5</v>
       </c>
       <c r="D12" s="19">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E12" s="22">
         <f t="shared" ref="E12:F12" si="5">E11-C12</f>
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F12" s="23">
         <f t="shared" si="5"/>
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
@@ -1699,18 +1699,18 @@
         <v>7</v>
       </c>
       <c r="C13" s="18">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D13" s="19">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E13" s="22">
         <f t="shared" ref="E13:F13" si="6">E12-C13</f>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F13" s="23">
         <f t="shared" si="6"/>
-        <v>60</v>
+        <v>11</v>
       </c>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
@@ -1739,18 +1739,18 @@
         <v>8</v>
       </c>
       <c r="C14" s="18">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D14" s="19">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E14" s="22">
         <f t="shared" ref="E14:F14" si="7">E13-C14</f>
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F14" s="23">
         <f t="shared" si="7"/>
-        <v>60</v>
+        <v>9</v>
       </c>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
@@ -1779,10 +1779,10 @@
         <v>9</v>
       </c>
       <c r="C15" s="18">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D15" s="19">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E15" s="22">
         <f t="shared" ref="E15:F15" si="8">E14-C15</f>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="F15" s="23">
         <f t="shared" si="8"/>
-        <v>60</v>
+        <v>6</v>
       </c>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
@@ -1819,18 +1819,18 @@
         <v>10</v>
       </c>
       <c r="C16" s="18">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D16" s="19">
         <v>0</v>
       </c>
       <c r="E16" s="22">
         <f t="shared" ref="E16:F16" si="9">E15-C16</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F16" s="23">
         <f t="shared" si="9"/>
-        <v>60</v>
+        <v>6</v>
       </c>
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
@@ -1859,18 +1859,18 @@
         <v>11</v>
       </c>
       <c r="C17" s="18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" s="24">
         <v>0</v>
       </c>
       <c r="E17" s="22">
         <f t="shared" ref="E17:F17" si="10">E16-C17</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" s="23">
         <f t="shared" si="10"/>
-        <v>60</v>
+        <v>6</v>
       </c>
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
@@ -1899,7 +1899,7 @@
         <v>12</v>
       </c>
       <c r="C18" s="18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D18" s="19">
         <v>0</v>
@@ -1910,7 +1910,7 @@
       </c>
       <c r="F18" s="23">
         <f t="shared" si="11"/>
-        <v>60</v>
+        <v>6</v>
       </c>
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
@@ -1935,17 +1935,23 @@
     </row>
     <row r="19" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3">
-        <f>SUM(C6:C18)</f>
-        <v>60</v>
-      </c>
-      <c r="D19" s="3">
-        <f>SUM(D6:D18)</f>
+      <c r="B19" s="17">
+        <v>13</v>
+      </c>
+      <c r="C19" s="18">
         <v>0</v>
       </c>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
+      <c r="D19" s="19">
+        <v>0</v>
+      </c>
+      <c r="E19" s="22">
+        <f t="shared" ref="E19" si="12">E18-C19</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="23">
+        <f t="shared" ref="F19" si="13">F18-D19</f>
+        <v>6</v>
+      </c>
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
@@ -1965,8 +1971,6 @@
     <row r="20" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
@@ -2263,8 +2267,14 @@
     <row r="31" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.6">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
-      <c r="C31" s="1"/>
-      <c r="D31" s="1"/>
+      <c r="C31" s="3">
+        <f>SUM(C7:C19)</f>
+        <v>60</v>
+      </c>
+      <c r="D31" s="3">
+        <f>SUM(D7:D19)</f>
+        <v>54</v>
+      </c>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
       <c r="G31" s="3"/>

</xml_diff>